<commit_message>
Added and Fixed a Lot of Things
</commit_message>
<xml_diff>
--- a/backend/utils/Template.xlsx
+++ b/backend/utils/Template.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B5A164-FBCF-4AFB-9CDA-AE923BFD5EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="1800" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="1" r:id="rId1"/>
@@ -2085,68 +2085,28 @@
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="7" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2158,7 +2118,16 @@
     <xf numFmtId="0" fontId="18" fillId="7" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2176,30 +2145,60 @@
     <xf numFmtId="0" fontId="18" fillId="7" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="89" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="99" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2213,11 +2212,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2814,33 +2814,33 @@
         <v>8</v>
       </c>
       <c r="E10" s="3"/>
-      <c r="G10" s="181" t="s">
+      <c r="G10" s="191" t="s">
         <v>9</v>
       </c>
-      <c r="H10" s="182"/>
-      <c r="I10" s="182"/>
-      <c r="J10" s="182"/>
-      <c r="K10" s="182"/>
-      <c r="L10" s="182"/>
-      <c r="M10" s="183"/>
+      <c r="H10" s="181"/>
+      <c r="I10" s="181"/>
+      <c r="J10" s="181"/>
+      <c r="K10" s="181"/>
+      <c r="L10" s="181"/>
+      <c r="M10" s="182"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G11" s="184" t="s">
+      <c r="G11" s="183" t="s">
         <v>10</v>
       </c>
-      <c r="H11" s="185"/>
-      <c r="I11" s="186"/>
-      <c r="K11" s="187" t="s">
+      <c r="H11" s="184"/>
+      <c r="I11" s="185"/>
+      <c r="K11" s="186" t="s">
         <v>11</v>
       </c>
-      <c r="L11" s="185"/>
-      <c r="M11" s="188"/>
+      <c r="L11" s="184"/>
+      <c r="M11" s="187"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="D12" s="189" t="s">
+      <c r="D12" s="177" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="173"/>
+      <c r="E12" s="123"/>
       <c r="G12" s="4"/>
       <c r="H12" s="5" t="s">
         <v>4</v>
@@ -2936,16 +2936,16 @@
       <c r="E17" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="G17" s="177" t="s">
+      <c r="G17" s="178" t="s">
         <v>19</v>
       </c>
-      <c r="H17" s="128"/>
-      <c r="I17" s="153"/>
-      <c r="K17" s="190" t="s">
+      <c r="H17" s="132"/>
+      <c r="I17" s="133"/>
+      <c r="K17" s="179" t="s">
         <v>20</v>
       </c>
-      <c r="L17" s="128"/>
-      <c r="M17" s="129"/>
+      <c r="L17" s="132"/>
+      <c r="M17" s="164"/>
     </row>
     <row r="18" spans="4:14" x14ac:dyDescent="0.25">
       <c r="D18" s="7">
@@ -3035,32 +3035,32 @@
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
       <c r="F24" s="13"/>
-      <c r="G24" s="191" t="s">
+      <c r="G24" s="180" t="s">
         <v>22</v>
       </c>
-      <c r="H24" s="182"/>
-      <c r="I24" s="182"/>
-      <c r="J24" s="182"/>
-      <c r="K24" s="182"/>
-      <c r="L24" s="182"/>
-      <c r="M24" s="183"/>
+      <c r="H24" s="181"/>
+      <c r="I24" s="181"/>
+      <c r="J24" s="181"/>
+      <c r="K24" s="181"/>
+      <c r="L24" s="181"/>
+      <c r="M24" s="182"/>
       <c r="N24" s="13"/>
     </row>
     <row r="25" spans="4:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
       <c r="F25" s="13"/>
-      <c r="G25" s="184" t="s">
+      <c r="G25" s="183" t="s">
         <v>23</v>
       </c>
-      <c r="H25" s="185"/>
-      <c r="I25" s="186"/>
+      <c r="H25" s="184"/>
+      <c r="I25" s="185"/>
       <c r="J25" s="14"/>
-      <c r="K25" s="187" t="s">
+      <c r="K25" s="186" t="s">
         <v>24</v>
       </c>
-      <c r="L25" s="185"/>
-      <c r="M25" s="188"/>
+      <c r="L25" s="184"/>
+      <c r="M25" s="187"/>
       <c r="N25" s="13"/>
     </row>
     <row r="26" spans="4:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3152,14 +3152,14 @@
       <c r="D31" s="13"/>
       <c r="E31" s="13"/>
       <c r="F31" s="13"/>
-      <c r="G31" s="177" t="s">
+      <c r="G31" s="178" t="s">
         <v>25</v>
       </c>
-      <c r="H31" s="128"/>
-      <c r="I31" s="153"/>
-      <c r="K31" s="178"/>
-      <c r="L31" s="179"/>
-      <c r="M31" s="180"/>
+      <c r="H31" s="132"/>
+      <c r="I31" s="133"/>
+      <c r="K31" s="188"/>
+      <c r="L31" s="189"/>
+      <c r="M31" s="190"/>
       <c r="N31" s="13"/>
     </row>
     <row r="32" spans="4:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4465,17 +4465,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="x30mJtPuYGTV7Z72zVyJ+KRnlHVZpTTmyXBT15aa+U+syNJJ0ki8fOkK2d98gCGENoLl4X4LoIL0/mh2EKzv+Q==" saltValue="ZkwyJaMIZSVSRCf3UNHWLQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="11">
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="K31:M31"/>
+    <mergeCell ref="G10:M10"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="K11:M11"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="G17:I17"/>
     <mergeCell ref="K17:M17"/>
     <mergeCell ref="G24:M24"/>
     <mergeCell ref="G25:I25"/>
     <mergeCell ref="K25:M25"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="K31:M31"/>
-    <mergeCell ref="G10:M10"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="K11:M11"/>
   </mergeCells>
   <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -4593,18 +4593,18 @@
       <c r="Z3" s="29"/>
     </row>
     <row r="4" spans="1:26" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="127" t="s">
+      <c r="A4" s="163" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="128"/>
-      <c r="C4" s="128"/>
-      <c r="D4" s="128"/>
-      <c r="E4" s="128"/>
-      <c r="F4" s="128"/>
-      <c r="G4" s="128"/>
-      <c r="H4" s="128"/>
-      <c r="I4" s="128"/>
-      <c r="J4" s="129"/>
+      <c r="B4" s="132"/>
+      <c r="C4" s="132"/>
+      <c r="D4" s="132"/>
+      <c r="E4" s="132"/>
+      <c r="F4" s="132"/>
+      <c r="G4" s="132"/>
+      <c r="H4" s="132"/>
+      <c r="I4" s="132"/>
+      <c r="J4" s="164"/>
       <c r="K4" s="29"/>
       <c r="L4" s="29"/>
       <c r="M4" s="29"/>
@@ -4858,19 +4858,19 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="46"/>
-      <c r="B13" s="130" t="s">
+      <c r="B13" s="165" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="128"/>
-      <c r="D13" s="128"/>
-      <c r="E13" s="129"/>
-      <c r="F13" s="131" t="s">
+      <c r="C13" s="132"/>
+      <c r="D13" s="132"/>
+      <c r="E13" s="164"/>
+      <c r="F13" s="166" t="s">
         <v>40</v>
       </c>
-      <c r="G13" s="128"/>
-      <c r="H13" s="128"/>
-      <c r="I13" s="128"/>
-      <c r="J13" s="129"/>
+      <c r="G13" s="132"/>
+      <c r="H13" s="132"/>
+      <c r="I13" s="132"/>
+      <c r="J13" s="164"/>
       <c r="K13" s="29"/>
       <c r="L13" s="29"/>
       <c r="M13" s="29"/>
@@ -4892,19 +4892,19 @@
       <c r="A14" s="47" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="132" t="s">
+      <c r="B14" s="167" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="133"/>
-      <c r="D14" s="133"/>
-      <c r="E14" s="134"/>
-      <c r="F14" s="132" t="s">
+      <c r="C14" s="168"/>
+      <c r="D14" s="168"/>
+      <c r="E14" s="128"/>
+      <c r="F14" s="167" t="s">
         <v>43</v>
       </c>
-      <c r="G14" s="133"/>
-      <c r="H14" s="133"/>
-      <c r="I14" s="133"/>
-      <c r="J14" s="134"/>
+      <c r="G14" s="168"/>
+      <c r="H14" s="168"/>
+      <c r="I14" s="168"/>
+      <c r="J14" s="128"/>
       <c r="K14" s="29"/>
       <c r="L14" s="29"/>
       <c r="M14" s="29"/>
@@ -4923,28 +4923,28 @@
       <c r="Z14" s="29"/>
     </row>
     <row r="15" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="135" t="s">
+      <c r="A15" s="169" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="137" t="s">
+      <c r="B15" s="171" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="137" t="s">
+      <c r="C15" s="171" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="137" t="s">
+      <c r="D15" s="171" t="s">
         <v>47</v>
       </c>
-      <c r="E15" s="137" t="s">
+      <c r="E15" s="171" t="s">
         <v>48</v>
       </c>
-      <c r="F15" s="139" t="s">
+      <c r="F15" s="173" t="s">
         <v>49</v>
       </c>
-      <c r="G15" s="122"/>
-      <c r="H15" s="122"/>
-      <c r="I15" s="140"/>
-      <c r="J15" s="141" t="s">
+      <c r="G15" s="161"/>
+      <c r="H15" s="161"/>
+      <c r="I15" s="174"/>
+      <c r="J15" s="175" t="s">
         <v>50</v>
       </c>
       <c r="K15" s="29"/>
@@ -4965,11 +4965,11 @@
       <c r="Z15" s="29"/>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A16" s="136"/>
-      <c r="B16" s="138"/>
-      <c r="C16" s="138"/>
-      <c r="D16" s="138"/>
-      <c r="E16" s="138"/>
+      <c r="A16" s="170"/>
+      <c r="B16" s="172"/>
+      <c r="C16" s="172"/>
+      <c r="D16" s="172"/>
+      <c r="E16" s="172"/>
       <c r="F16" s="48" t="s">
         <v>51</v>
       </c>
@@ -4982,7 +4982,7 @@
       <c r="I16" s="49" t="s">
         <v>54</v>
       </c>
-      <c r="J16" s="142"/>
+      <c r="J16" s="176"/>
       <c r="K16" s="29"/>
       <c r="L16" s="29"/>
       <c r="M16" s="29"/>
@@ -5001,18 +5001,18 @@
       <c r="Z16" s="29"/>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A17" s="121" t="s">
+      <c r="A17" s="160" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="122"/>
-      <c r="F17" s="122"/>
-      <c r="G17" s="122"/>
-      <c r="H17" s="122"/>
-      <c r="I17" s="122"/>
-      <c r="J17" s="123"/>
+      <c r="B17" s="161"/>
+      <c r="C17" s="161"/>
+      <c r="D17" s="161"/>
+      <c r="E17" s="161"/>
+      <c r="F17" s="161"/>
+      <c r="G17" s="161"/>
+      <c r="H17" s="161"/>
+      <c r="I17" s="161"/>
+      <c r="J17" s="155"/>
       <c r="K17" s="29"/>
       <c r="L17" s="29"/>
       <c r="M17" s="29"/>
@@ -5031,13 +5031,13 @@
       <c r="Z17" s="29"/>
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A18" s="124" t="s">
+      <c r="A18" s="162" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="125"/>
-      <c r="C18" s="125"/>
-      <c r="D18" s="125"/>
-      <c r="E18" s="126"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="130"/>
       <c r="F18" s="50"/>
       <c r="G18" s="50"/>
       <c r="H18" s="50"/>
@@ -5280,13 +5280,13 @@
       <c r="Z25" s="29"/>
     </row>
     <row r="26" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="143" t="s">
+      <c r="A26" s="141" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="144"/>
-      <c r="C26" s="144"/>
-      <c r="D26" s="144"/>
-      <c r="E26" s="145"/>
+      <c r="B26" s="142"/>
+      <c r="C26" s="142"/>
+      <c r="D26" s="142"/>
+      <c r="E26" s="143"/>
       <c r="F26" s="66"/>
       <c r="G26" s="66"/>
       <c r="H26" s="66"/>
@@ -5370,13 +5370,13 @@
       <c r="Z28" s="29"/>
     </row>
     <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="143" t="s">
+      <c r="A29" s="141" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="144"/>
-      <c r="C29" s="144"/>
-      <c r="D29" s="144"/>
-      <c r="E29" s="145"/>
+      <c r="B29" s="142"/>
+      <c r="C29" s="142"/>
+      <c r="D29" s="142"/>
+      <c r="E29" s="143"/>
       <c r="F29" s="66"/>
       <c r="G29" s="66"/>
       <c r="H29" s="66"/>
@@ -5490,13 +5490,13 @@
       <c r="Z32" s="29"/>
     </row>
     <row r="33" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="146" t="s">
+      <c r="A33" s="158" t="s">
         <v>71</v>
       </c>
-      <c r="B33" s="147"/>
-      <c r="C33" s="147"/>
-      <c r="D33" s="147"/>
-      <c r="E33" s="148"/>
+      <c r="B33" s="138"/>
+      <c r="C33" s="138"/>
+      <c r="D33" s="138"/>
+      <c r="E33" s="159"/>
       <c r="F33" s="66"/>
       <c r="G33" s="66"/>
       <c r="H33" s="66"/>
@@ -5550,13 +5550,13 @@
       <c r="Z34" s="29"/>
     </row>
     <row r="35" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="143" t="s">
+      <c r="A35" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="144"/>
-      <c r="C35" s="144"/>
-      <c r="D35" s="144"/>
-      <c r="E35" s="145"/>
+      <c r="B35" s="142"/>
+      <c r="C35" s="142"/>
+      <c r="D35" s="142"/>
+      <c r="E35" s="143"/>
       <c r="F35" s="66"/>
       <c r="G35" s="66"/>
       <c r="H35" s="66"/>
@@ -5610,13 +5610,13 @@
       <c r="Z36" s="29"/>
     </row>
     <row r="37" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="146" t="s">
+      <c r="A37" s="158" t="s">
         <v>75</v>
       </c>
-      <c r="B37" s="147"/>
-      <c r="C37" s="147"/>
-      <c r="D37" s="147"/>
-      <c r="E37" s="148"/>
+      <c r="B37" s="138"/>
+      <c r="C37" s="138"/>
+      <c r="D37" s="138"/>
+      <c r="E37" s="159"/>
       <c r="F37" s="66"/>
       <c r="G37" s="66"/>
       <c r="H37" s="66"/>
@@ -5670,18 +5670,18 @@
       <c r="Z38" s="29"/>
     </row>
     <row r="39" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="149" t="s">
+      <c r="A39" s="140" t="s">
         <v>77</v>
       </c>
-      <c r="B39" s="125"/>
-      <c r="C39" s="125"/>
-      <c r="D39" s="125"/>
-      <c r="E39" s="125"/>
-      <c r="F39" s="125"/>
-      <c r="G39" s="125"/>
-      <c r="H39" s="125"/>
-      <c r="I39" s="125"/>
-      <c r="J39" s="150"/>
+      <c r="B39" s="122"/>
+      <c r="C39" s="122"/>
+      <c r="D39" s="122"/>
+      <c r="E39" s="122"/>
+      <c r="F39" s="122"/>
+      <c r="G39" s="122"/>
+      <c r="H39" s="122"/>
+      <c r="I39" s="122"/>
+      <c r="J39" s="124"/>
       <c r="K39" s="29"/>
       <c r="L39" s="29"/>
       <c r="M39" s="29"/>
@@ -5700,13 +5700,13 @@
       <c r="Z39" s="29"/>
     </row>
     <row r="40" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="151" t="s">
+      <c r="A40" s="129" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="125"/>
-      <c r="C40" s="125"/>
-      <c r="D40" s="125"/>
-      <c r="E40" s="126"/>
+      <c r="B40" s="122"/>
+      <c r="C40" s="122"/>
+      <c r="D40" s="122"/>
+      <c r="E40" s="130"/>
       <c r="F40" s="50"/>
       <c r="G40" s="50"/>
       <c r="H40" s="50"/>
@@ -5940,18 +5940,18 @@
       <c r="Z47" s="29"/>
     </row>
     <row r="48" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="149" t="s">
+      <c r="A48" s="140" t="s">
         <v>86</v>
       </c>
-      <c r="B48" s="125"/>
-      <c r="C48" s="125"/>
-      <c r="D48" s="125"/>
-      <c r="E48" s="125"/>
-      <c r="F48" s="125"/>
-      <c r="G48" s="125"/>
-      <c r="H48" s="125"/>
-      <c r="I48" s="125"/>
-      <c r="J48" s="150"/>
+      <c r="B48" s="122"/>
+      <c r="C48" s="122"/>
+      <c r="D48" s="122"/>
+      <c r="E48" s="122"/>
+      <c r="F48" s="122"/>
+      <c r="G48" s="122"/>
+      <c r="H48" s="122"/>
+      <c r="I48" s="122"/>
+      <c r="J48" s="124"/>
       <c r="K48" s="29"/>
       <c r="L48" s="29"/>
       <c r="M48" s="29"/>
@@ -5970,13 +5970,13 @@
       <c r="Z48" s="29"/>
     </row>
     <row r="49" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="143" t="s">
+      <c r="A49" s="141" t="s">
         <v>87</v>
       </c>
-      <c r="B49" s="144"/>
-      <c r="C49" s="144"/>
-      <c r="D49" s="144"/>
-      <c r="E49" s="145"/>
+      <c r="B49" s="142"/>
+      <c r="C49" s="142"/>
+      <c r="D49" s="142"/>
+      <c r="E49" s="143"/>
       <c r="F49" s="50"/>
       <c r="G49" s="50"/>
       <c r="H49" s="50"/>
@@ -6150,18 +6150,18 @@
       <c r="Z54" s="29"/>
     </row>
     <row r="55" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="149" t="s">
+      <c r="A55" s="140" t="s">
         <v>93</v>
       </c>
-      <c r="B55" s="125"/>
-      <c r="C55" s="125"/>
-      <c r="D55" s="125"/>
-      <c r="E55" s="125"/>
-      <c r="F55" s="125"/>
-      <c r="G55" s="125"/>
-      <c r="H55" s="125"/>
-      <c r="I55" s="125"/>
-      <c r="J55" s="150"/>
+      <c r="B55" s="122"/>
+      <c r="C55" s="122"/>
+      <c r="D55" s="122"/>
+      <c r="E55" s="122"/>
+      <c r="F55" s="122"/>
+      <c r="G55" s="122"/>
+      <c r="H55" s="122"/>
+      <c r="I55" s="122"/>
+      <c r="J55" s="124"/>
       <c r="K55" s="29"/>
       <c r="L55" s="29"/>
       <c r="M55" s="29"/>
@@ -6180,13 +6180,13 @@
       <c r="Z55" s="29"/>
     </row>
     <row r="56" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="151" t="s">
+      <c r="A56" s="129" t="s">
         <v>94</v>
       </c>
-      <c r="B56" s="125"/>
-      <c r="C56" s="125"/>
-      <c r="D56" s="125"/>
-      <c r="E56" s="126"/>
+      <c r="B56" s="122"/>
+      <c r="C56" s="122"/>
+      <c r="D56" s="122"/>
+      <c r="E56" s="130"/>
       <c r="F56" s="79"/>
       <c r="G56" s="79"/>
       <c r="H56" s="79"/>
@@ -6240,13 +6240,13 @@
       <c r="Z57" s="29"/>
     </row>
     <row r="58" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="151" t="s">
+      <c r="A58" s="129" t="s">
         <v>96</v>
       </c>
-      <c r="B58" s="125"/>
-      <c r="C58" s="125"/>
-      <c r="D58" s="125"/>
-      <c r="E58" s="126"/>
+      <c r="B58" s="122"/>
+      <c r="C58" s="122"/>
+      <c r="D58" s="122"/>
+      <c r="E58" s="130"/>
       <c r="F58" s="61"/>
       <c r="G58" s="61"/>
       <c r="H58" s="61"/>
@@ -6300,13 +6300,13 @@
       <c r="Z59" s="29"/>
     </row>
     <row r="60" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="151" t="s">
+      <c r="A60" s="129" t="s">
         <v>98</v>
       </c>
-      <c r="B60" s="125"/>
-      <c r="C60" s="125"/>
-      <c r="D60" s="125"/>
-      <c r="E60" s="126"/>
+      <c r="B60" s="122"/>
+      <c r="C60" s="122"/>
+      <c r="D60" s="122"/>
+      <c r="E60" s="130"/>
       <c r="F60" s="66"/>
       <c r="G60" s="66"/>
       <c r="H60" s="66"/>
@@ -6360,13 +6360,13 @@
       <c r="Z61" s="29"/>
     </row>
     <row r="62" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="151" t="s">
+      <c r="A62" s="129" t="s">
         <v>99</v>
       </c>
-      <c r="B62" s="125"/>
-      <c r="C62" s="125"/>
-      <c r="D62" s="125"/>
-      <c r="E62" s="126"/>
+      <c r="B62" s="122"/>
+      <c r="C62" s="122"/>
+      <c r="D62" s="122"/>
+      <c r="E62" s="130"/>
       <c r="F62" s="66"/>
       <c r="G62" s="66"/>
       <c r="H62" s="66"/>
@@ -6420,13 +6420,13 @@
       <c r="Z63" s="29"/>
     </row>
     <row r="64" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="151" t="s">
+      <c r="A64" s="129" t="s">
         <v>101</v>
       </c>
-      <c r="B64" s="125"/>
-      <c r="C64" s="125"/>
-      <c r="D64" s="125"/>
-      <c r="E64" s="126"/>
+      <c r="B64" s="122"/>
+      <c r="C64" s="122"/>
+      <c r="D64" s="122"/>
+      <c r="E64" s="130"/>
       <c r="F64" s="66"/>
       <c r="G64" s="66"/>
       <c r="H64" s="66"/>
@@ -6480,13 +6480,13 @@
       <c r="Z65" s="29"/>
     </row>
     <row r="66" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="151" t="s">
+      <c r="A66" s="129" t="s">
         <v>102</v>
       </c>
-      <c r="B66" s="125"/>
-      <c r="C66" s="125"/>
-      <c r="D66" s="125"/>
-      <c r="E66" s="126"/>
+      <c r="B66" s="122"/>
+      <c r="C66" s="122"/>
+      <c r="D66" s="122"/>
+      <c r="E66" s="130"/>
       <c r="F66" s="66"/>
       <c r="G66" s="66"/>
       <c r="H66" s="66"/>
@@ -6540,13 +6540,13 @@
       <c r="Z67" s="29"/>
     </row>
     <row r="68" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="151" t="s">
+      <c r="A68" s="129" t="s">
         <v>104</v>
       </c>
-      <c r="B68" s="125"/>
-      <c r="C68" s="125"/>
-      <c r="D68" s="125"/>
-      <c r="E68" s="126"/>
+      <c r="B68" s="122"/>
+      <c r="C68" s="122"/>
+      <c r="D68" s="122"/>
+      <c r="E68" s="130"/>
       <c r="F68" s="84"/>
       <c r="G68" s="84"/>
       <c r="H68" s="84"/>
@@ -6600,17 +6600,17 @@
       <c r="Z69" s="29"/>
     </row>
     <row r="70" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="152" t="s">
+      <c r="A70" s="131" t="s">
         <v>106</v>
       </c>
-      <c r="B70" s="128"/>
-      <c r="C70" s="128"/>
-      <c r="D70" s="128"/>
-      <c r="E70" s="153"/>
+      <c r="B70" s="132"/>
+      <c r="C70" s="132"/>
+      <c r="D70" s="132"/>
+      <c r="E70" s="133"/>
       <c r="F70" s="89"/>
-      <c r="G70" s="154"/>
-      <c r="H70" s="125"/>
-      <c r="I70" s="126"/>
+      <c r="G70" s="134"/>
+      <c r="H70" s="122"/>
+      <c r="I70" s="130"/>
       <c r="J70" s="88"/>
       <c r="K70" s="29"/>
       <c r="L70" s="29"/>
@@ -6660,13 +6660,13 @@
       <c r="Z71" s="29"/>
     </row>
     <row r="72" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="151" t="s">
+      <c r="A72" s="129" t="s">
         <v>107</v>
       </c>
-      <c r="B72" s="125"/>
-      <c r="C72" s="125"/>
-      <c r="D72" s="125"/>
-      <c r="E72" s="126"/>
+      <c r="B72" s="122"/>
+      <c r="C72" s="122"/>
+      <c r="D72" s="122"/>
+      <c r="E72" s="130"/>
       <c r="F72" s="66"/>
       <c r="G72" s="66"/>
       <c r="H72" s="66"/>
@@ -6720,18 +6720,18 @@
       <c r="Z73" s="29"/>
     </row>
     <row r="74" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="149" t="s">
+      <c r="A74" s="140" t="s">
         <v>108</v>
       </c>
-      <c r="B74" s="125"/>
-      <c r="C74" s="125"/>
-      <c r="D74" s="125"/>
-      <c r="E74" s="125"/>
-      <c r="F74" s="125"/>
-      <c r="G74" s="125"/>
-      <c r="H74" s="125"/>
-      <c r="I74" s="125"/>
-      <c r="J74" s="150"/>
+      <c r="B74" s="122"/>
+      <c r="C74" s="122"/>
+      <c r="D74" s="122"/>
+      <c r="E74" s="122"/>
+      <c r="F74" s="122"/>
+      <c r="G74" s="122"/>
+      <c r="H74" s="122"/>
+      <c r="I74" s="122"/>
+      <c r="J74" s="124"/>
       <c r="K74" s="29"/>
       <c r="L74" s="29"/>
       <c r="M74" s="29"/>
@@ -6750,13 +6750,13 @@
       <c r="Z74" s="29"/>
     </row>
     <row r="75" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="143" t="s">
+      <c r="A75" s="141" t="s">
         <v>109</v>
       </c>
-      <c r="B75" s="144"/>
-      <c r="C75" s="144"/>
-      <c r="D75" s="144"/>
-      <c r="E75" s="145"/>
+      <c r="B75" s="142"/>
+      <c r="C75" s="142"/>
+      <c r="D75" s="142"/>
+      <c r="E75" s="143"/>
       <c r="F75" s="50"/>
       <c r="G75" s="50"/>
       <c r="H75" s="50"/>
@@ -7086,22 +7086,22 @@
       <c r="Z83" s="29"/>
     </row>
     <row r="84" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="159" t="s">
+      <c r="A84" s="144" t="s">
         <v>115</v>
       </c>
-      <c r="B84" s="160"/>
-      <c r="C84" s="160"/>
-      <c r="D84" s="160"/>
-      <c r="E84" s="161"/>
-      <c r="F84" s="165"/>
-      <c r="G84" s="166"/>
+      <c r="B84" s="145"/>
+      <c r="C84" s="145"/>
+      <c r="D84" s="145"/>
+      <c r="E84" s="146"/>
+      <c r="F84" s="150"/>
+      <c r="G84" s="151"/>
       <c r="H84" s="99" t="s">
         <v>116</v>
       </c>
-      <c r="I84" s="169" t="s">
+      <c r="I84" s="154" t="s">
         <v>117</v>
       </c>
-      <c r="J84" s="123"/>
+      <c r="J84" s="155"/>
       <c r="K84" s="29"/>
       <c r="L84" s="29"/>
       <c r="M84" s="29"/>
@@ -7120,19 +7120,19 @@
       <c r="Z84" s="29"/>
     </row>
     <row r="85" spans="1:26" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="162"/>
-      <c r="B85" s="163"/>
-      <c r="C85" s="163"/>
-      <c r="D85" s="163"/>
-      <c r="E85" s="164"/>
-      <c r="F85" s="167"/>
-      <c r="G85" s="168"/>
+      <c r="A85" s="147"/>
+      <c r="B85" s="148"/>
+      <c r="C85" s="148"/>
+      <c r="D85" s="148"/>
+      <c r="E85" s="149"/>
+      <c r="F85" s="152"/>
+      <c r="G85" s="153"/>
       <c r="H85" s="100"/>
-      <c r="I85" s="170" t="str">
+      <c r="I85" s="156" t="str">
         <f>IF(H85="","",LOOKUP(H85,ROUNDUP,DESCRIPTION))</f>
         <v/>
       </c>
-      <c r="J85" s="171"/>
+      <c r="J85" s="157"/>
       <c r="K85" s="29"/>
       <c r="L85" s="29"/>
       <c r="M85" s="29"/>
@@ -7188,21 +7188,21 @@
     </row>
     <row r="87" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="108"/>
-      <c r="B87" s="155" t="s">
+      <c r="B87" s="135" t="s">
         <v>39</v>
       </c>
-      <c r="C87" s="128"/>
-      <c r="D87" s="156"/>
-      <c r="E87" s="155" t="s">
+      <c r="C87" s="132"/>
+      <c r="D87" s="136"/>
+      <c r="E87" s="135" t="s">
         <v>122</v>
       </c>
-      <c r="F87" s="128"/>
-      <c r="G87" s="156"/>
-      <c r="H87" s="157" t="s">
+      <c r="F87" s="132"/>
+      <c r="G87" s="136"/>
+      <c r="H87" s="137" t="s">
         <v>40</v>
       </c>
-      <c r="I87" s="147"/>
-      <c r="J87" s="158"/>
+      <c r="I87" s="138"/>
+      <c r="J87" s="139"/>
       <c r="K87" s="29"/>
       <c r="L87" s="29"/>
       <c r="M87" s="29"/>
@@ -7224,21 +7224,21 @@
       <c r="A88" s="109" t="s">
         <v>123</v>
       </c>
-      <c r="B88" s="172" t="s">
+      <c r="B88" s="121" t="s">
         <v>42</v>
       </c>
-      <c r="C88" s="125"/>
-      <c r="D88" s="173"/>
-      <c r="E88" s="172" t="s">
+      <c r="C88" s="122"/>
+      <c r="D88" s="123"/>
+      <c r="E88" s="121" t="s">
         <v>124</v>
       </c>
-      <c r="F88" s="125"/>
-      <c r="G88" s="173"/>
-      <c r="H88" s="172" t="s">
+      <c r="F88" s="122"/>
+      <c r="G88" s="123"/>
+      <c r="H88" s="121" t="s">
         <v>125</v>
       </c>
-      <c r="I88" s="125"/>
-      <c r="J88" s="150"/>
+      <c r="I88" s="122"/>
+      <c r="J88" s="124"/>
       <c r="K88" s="29"/>
       <c r="L88" s="29"/>
       <c r="M88" s="29"/>
@@ -7263,8 +7263,8 @@
       <c r="B89" s="111" t="s">
         <v>126</v>
       </c>
-      <c r="C89" s="174"/>
-      <c r="D89" s="175"/>
+      <c r="C89" s="125"/>
+      <c r="D89" s="126"/>
       <c r="E89" s="111" t="s">
         <v>126</v>
       </c>
@@ -7273,8 +7273,8 @@
       <c r="H89" s="114" t="s">
         <v>126</v>
       </c>
-      <c r="I89" s="176"/>
-      <c r="J89" s="134"/>
+      <c r="I89" s="127"/>
+      <c r="J89" s="128"/>
       <c r="K89" s="29"/>
       <c r="L89" s="29"/>
       <c r="M89" s="29"/>
@@ -32803,11 +32803,35 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="48">
-    <mergeCell ref="B88:D88"/>
-    <mergeCell ref="E88:G88"/>
-    <mergeCell ref="H88:J88"/>
-    <mergeCell ref="C89:D89"/>
-    <mergeCell ref="I89:J89"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="F14:J14"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A39:J39"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A48:J48"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A55:J55"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A62:E62"/>
+    <mergeCell ref="A64:E64"/>
     <mergeCell ref="A66:E66"/>
     <mergeCell ref="A68:E68"/>
     <mergeCell ref="A70:E70"/>
@@ -32822,35 +32846,11 @@
     <mergeCell ref="F84:G85"/>
     <mergeCell ref="I84:J84"/>
     <mergeCell ref="I85:J85"/>
-    <mergeCell ref="A56:E56"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A62:E62"/>
-    <mergeCell ref="A64:E64"/>
-    <mergeCell ref="A39:J39"/>
-    <mergeCell ref="A40:E40"/>
-    <mergeCell ref="A48:J48"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A55:J55"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="F14:J14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="B88:D88"/>
+    <mergeCell ref="E88:G88"/>
+    <mergeCell ref="H88:J88"/>
+    <mergeCell ref="C89:D89"/>
+    <mergeCell ref="I89:J89"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>

</xml_diff>